<commit_message>
SHELF, SYSHECF, and other updates
</commit_message>
<xml_diff>
--- a/InputData/add-outputs/VoaSL/Value of a Statistical Life.xlsx
+++ b/InputData/add-outputs/VoaSL/Value of a Statistical Life.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreazafra/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rachel Goldstein\Desktop\EPS Models\Mexico EPS\InputData\add-outputs\VoaSL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{6E7A770A-7C28-0545-8D7C-1EB6139DDDB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C07C382-D83B-4BDF-89DC-90D091D010E7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A83E6DD-4F75-48CB-A65F-FC37C57EBF1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="35080" yWindow="2640" windowWidth="27000" windowHeight="18160" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="44145" yWindow="1230" windowWidth="22785" windowHeight="14115" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -147,7 +147,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -214,11 +214,11 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="2" builtinId="3"/>
@@ -526,17 +526,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B37"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="38.28515625" customWidth="1"/>
+    <col min="2" max="2" width="38.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -544,75 +544,75 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>0.97135205460935392</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>0.84730412960844359</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>14</v>
       </c>
@@ -620,7 +620,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>2006</v>
       </c>
@@ -628,7 +628,7 @@
         <v>10.901017260273969</v>
       </c>
     </row>
-    <row r="22" spans="1:2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>2007</v>
       </c>
@@ -636,7 +636,7 @@
         <v>10.926903013698627</v>
       </c>
     </row>
-    <row r="23" spans="1:2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>2008</v>
       </c>
@@ -644,7 +644,7 @@
         <v>11.138301912568313</v>
       </c>
     </row>
-    <row r="24" spans="1:2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>2009</v>
       </c>
@@ -652,7 +652,7 @@
         <v>13.509501369863028</v>
       </c>
     </row>
-    <row r="25" spans="1:2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>2010</v>
       </c>
@@ -660,7 +660,7 @@
         <v>12.636678082191793</v>
       </c>
     </row>
-    <row r="26" spans="1:2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>2011</v>
       </c>
@@ -668,7 +668,7 @@
         <v>12.427292876712329</v>
       </c>
     </row>
-    <row r="27" spans="1:2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>2012</v>
       </c>
@@ -676,7 +676,7 @@
         <v>13.168531967213106</v>
       </c>
     </row>
-    <row r="28" spans="1:2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>2013</v>
       </c>
@@ -684,7 +684,7 @@
         <v>12.767464383561641</v>
       </c>
     </row>
-    <row r="29" spans="1:2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>2014</v>
       </c>
@@ -692,7 +692,7 @@
         <v>13.298290410958895</v>
       </c>
     </row>
-    <row r="30" spans="1:2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>2015</v>
       </c>
@@ -700,7 +700,7 @@
         <v>15.854175890410984</v>
       </c>
     </row>
-    <row r="31" spans="1:2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>2016</v>
       </c>
@@ -708,7 +708,7 @@
         <v>18.656701092896164</v>
       </c>
     </row>
-    <row r="32" spans="1:2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>2017</v>
       </c>
@@ -716,7 +716,7 @@
         <v>18.929111232876703</v>
       </c>
     </row>
-    <row r="33" spans="1:2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>2018</v>
       </c>
@@ -724,7 +724,7 @@
         <v>18.822825165562914</v>
       </c>
     </row>
-    <row r="34" spans="1:2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>2019</v>
       </c>
@@ -732,7 +732,7 @@
         <v>19.260525900000001</v>
       </c>
     </row>
-    <row r="35" spans="1:2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>2020</v>
       </c>
@@ -740,7 +740,7 @@
         <v>21.493461509999999</v>
       </c>
     </row>
-    <row r="36" spans="1:2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>2021</v>
       </c>
@@ -748,7 +748,7 @@
         <v>20.280012648221323</v>
       </c>
     </row>
-    <row r="37" spans="1:2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>12</v>
       </c>
@@ -762,20 +762,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="43.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" customWidth="1"/>
-    <col min="4" max="4" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.33203125" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" customWidth="1"/>
+    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -783,7 +783,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -791,7 +791,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -799,21 +799,21 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="95.25" customHeight="1">
-      <c r="B7" s="10" t="s">
+    <row r="7" spans="1:6" ht="95.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C9" t="s">
         <v>22</v>
       </c>
@@ -827,7 +827,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>26</v>
       </c>
@@ -846,7 +846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>27</v>
       </c>
@@ -864,7 +864,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>28</v>
       </c>
@@ -883,7 +883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C14" t="s">
         <v>29</v>
       </c>
@@ -891,14 +891,14 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>30</v>
       </c>
       <c r="C15" s="6">
         <v>2000000</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="8">
         <f>C15*About!A16</f>
         <v>1694608.2592168872</v>
       </c>
@@ -924,21 +924,21 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="16.42578125" customWidth="1"/>
+    <col min="1" max="2" width="16.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B1" s="4" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>32</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="10">
         <f>Mexico!D15</f>
         <v>1694608.2592168872</v>
       </c>
@@ -949,6 +949,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -1092,29 +1107,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DA52DC3-B7BC-4D08-8BBD-9D6D8AD2E73D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8A4A89-CB37-46A1-B23B-360F77ABB45F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55E723E2-6DC7-4512-B42B-913F6DC408F1}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8A4A89-CB37-46A1-B23B-360F77ABB45F}"/>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DA52DC3-B7BC-4D08-8BBD-9D6D8AD2E73D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55E723E2-6DC7-4512-B42B-913F6DC408F1}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>